<commit_message>
Mise à jour Contact, Veille et tableau
</commit_message>
<xml_diff>
--- a/src/assets/Tableau_Abdoulaye_Final.xlsx
+++ b/src/assets/Tableau_Abdoulaye_Final.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abdcsko/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abdcsko/Documents/portfolio/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{182D5723-A0C7-C949-AE70-3AB4AAAE13F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA188761-EA21-FD4E-B679-4D35A4E8A59D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,9 +37,6 @@
     <t>NOM et prénom : Cissokho Abdoulaye</t>
   </si>
   <si>
-    <t xml:space="preserve">N° candidat : </t>
-  </si>
-  <si>
     <t>Centre de formation : EFREI</t>
   </si>
   <si>
@@ -50,9 +47,6 @@
   </si>
   <si>
     <t>X SLAM</t>
-  </si>
-  <si>
-    <t>Adresse URL du portfolio : https://portfolio-abd-x4vj.vercel.app/</t>
   </si>
   <si>
     <t>Compétences mises en œuvre
@@ -276,6 +270,12 @@
     <t>23/04/26
 au
 16/05/26</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://portfolio-abd-ben3.vercel.app/</t>
+  </si>
+  <si>
+    <t>N° candidat : 2303834866</t>
   </si>
 </sst>
 </file>
@@ -709,11 +709,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -737,17 +748,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Euro" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -1068,147 +1068,147 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="33" t="s">
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="34"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="1:13" ht="41" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="22" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="23"/>
-      <c r="H3" s="24"/>
+      <c r="B3" s="28"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="28"/>
+      <c r="H3" s="29"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="37" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="H4" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="12" t="s">
+    </row>
+    <row r="5" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="26"/>
+    </row>
+    <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="34" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="35" t="s">
+      <c r="B6" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="37"/>
-    </row>
-    <row r="6" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="29" t="s">
+      <c r="C6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="D6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="6" t="s">
+    </row>
+    <row r="7" spans="1:13" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="35"/>
+      <c r="B7" s="31"/>
+      <c r="C7" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="30"/>
-      <c r="B7" s="26"/>
-      <c r="C7" s="8" t="s">
+      <c r="E7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="G7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="H7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="8" t="s">
+    </row>
+    <row r="8" spans="1:13" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="27" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="33"/>
     </row>
     <row r="9" spans="1:13" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
@@ -1218,13 +1218,13 @@
     </row>
     <row r="10" spans="1:13" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
@@ -1234,44 +1234,44 @@
     </row>
     <row r="11" spans="1:13" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H11" s="16"/>
     </row>
     <row r="12" spans="1:13" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
     </row>
     <row r="13" spans="1:13" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -1279,15 +1279,15 @@
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
       <c r="H13" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:13" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
@@ -1295,15 +1295,15 @@
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
       <c r="H14" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:13" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="13" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
@@ -1311,15 +1311,15 @@
       <c r="F15" s="16"/>
       <c r="G15" s="16"/>
       <c r="H15" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:13" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
@@ -1327,20 +1327,20 @@
       <c r="F16" s="16"/>
       <c r="G16" s="16"/>
       <c r="H16" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="16"/>
@@ -1348,42 +1348,42 @@
     </row>
     <row r="18" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="13" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C18" s="16"/>
       <c r="D18" s="15"/>
       <c r="E18" s="16"/>
       <c r="F18" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
     </row>
     <row r="19" spans="1:8" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A19" s="19" t="s">
-        <v>40</v>
-      </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="21"/>
+      <c r="A19" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="23"/>
     </row>
     <row r="20" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="13" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C20" s="16"/>
       <c r="D20" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
@@ -1392,16 +1392,16 @@
     </row>
     <row r="21" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E21" s="16"/>
       <c r="F21" s="16"/>
@@ -1420,52 +1420,52 @@
     </row>
     <row r="23" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="16"/>
       <c r="F23" s="16"/>
       <c r="G23" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="13" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C24" s="16"/>
       <c r="D24" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E24" s="16"/>
       <c r="F24" s="16"/>
       <c r="G24" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H24" s="16"/>
     </row>
     <row r="25" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="13" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="16"/>
       <c r="F25" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
@@ -1481,64 +1481,64 @@
       <c r="H26" s="16"/>
     </row>
     <row r="27" spans="1:8" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="21"/>
+      <c r="A27" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="23"/>
     </row>
     <row r="28" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
       <c r="F28" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H28" s="16"/>
     </row>
     <row r="29" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E29" s="16"/>
       <c r="F29" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H29" s="16"/>
     </row>
     <row r="30" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
@@ -1548,15 +1548,15 @@
     </row>
     <row r="31" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
       <c r="E31" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F31" s="16"/>
       <c r="G31" s="16"/>
@@ -1564,15 +1564,15 @@
     </row>
     <row r="32" spans="1:8" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F32" s="16"/>
       <c r="G32" s="16"/>
@@ -1610,11 +1610,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A5:H5"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="F3:H3"/>
     <mergeCell ref="B6:B7"/>
@@ -1622,6 +1617,11 @@
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>

</xml_diff>